<commit_message>
starting a fast  api study
</commit_message>
<xml_diff>
--- a/dsa_top_problems.xlsx
+++ b/dsa_top_problems.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sande\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sande\OneDrive\Desktop\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2BAE9D-B9CD-459C-AD04-A5534E1FF415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA55AEFD-1568-41B3-9F40-C1BCD2441CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="210">
   <si>
     <t>🚀  DSA Interview Prep — Top Company-Asked Problems</t>
   </si>
@@ -628,7 +628,34 @@
     <t>✅</t>
   </si>
   <si>
-    <t xml:space="preserve">set(nums)` internally goes through **every element once** to build the set. So it's still O(n). The `len()` check is O(1) — instant </t>
+    <t>HashMap (key value storage)</t>
+  </si>
+  <si>
+    <t>Sliding Window(dynamic subarray range)</t>
+  </si>
+  <si>
+    <t>HashSet (unique elements only)</t>
+  </si>
+  <si>
+    <t>Prefix Sum(cumulative sum array)</t>
+  </si>
+  <si>
+    <t>Kadane's DP (max subarray sum)</t>
+  </si>
+  <si>
+    <t>DP(Dynamic Programming) → reuse subproblems</t>
+  </si>
+  <si>
+    <t>Binary Search (Search sorted array)</t>
+  </si>
+  <si>
+    <t>Two Pointers (left right indices)</t>
+  </si>
+  <si>
+    <t>Expand Around Center (palindrome center expand)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Its Dificult problem for me to solve </t>
   </si>
 </sst>
 </file>
@@ -1361,7 +1388,7 @@
       <c r="J4" s="25"/>
       <c r="K4" s="25"/>
     </row>
-    <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="26.4" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>199</v>
       </c>
@@ -1374,8 +1401,8 @@
       <c r="D5" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>17</v>
+      <c r="E5" s="18" t="s">
+        <v>200</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>18</v>
@@ -1394,7 +1421,7 @@
       </c>
       <c r="K5" s="16"/>
     </row>
-    <row r="6" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="23" t="s">
         <v>199</v>
       </c>
@@ -1407,8 +1434,8 @@
       <c r="D6" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="16" t="s">
-        <v>24</v>
+      <c r="E6" s="18" t="s">
+        <v>201</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>18</v>
@@ -1427,7 +1454,7 @@
       </c>
       <c r="K6" s="16"/>
     </row>
-    <row r="7" spans="1:11" ht="66" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="26.4" x14ac:dyDescent="0.35">
       <c r="A7" s="23" t="s">
         <v>199</v>
       </c>
@@ -1440,8 +1467,8 @@
       <c r="D7" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>28</v>
+      <c r="E7" s="18" t="s">
+        <v>202</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>18</v>
@@ -1458,11 +1485,9 @@
       <c r="J7" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="K7" s="18" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K7" s="18"/>
+    </row>
+    <row r="8" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="23" t="s">
         <v>14</v>
       </c>
@@ -1475,8 +1500,8 @@
       <c r="D8" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>32</v>
+      <c r="E8" s="18" t="s">
+        <v>203</v>
       </c>
       <c r="F8" s="20" t="s">
         <v>33</v>
@@ -1493,11 +1518,13 @@
       <c r="J8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="16"/>
-    </row>
-    <row r="9" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K8" s="16" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="33.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
-        <v>14</v>
+        <v>199</v>
       </c>
       <c r="B9" s="13">
         <v>5</v>
@@ -1508,8 +1535,8 @@
       <c r="D9" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>37</v>
+      <c r="E9" s="18" t="s">
+        <v>204</v>
       </c>
       <c r="F9" s="20" t="s">
         <v>33</v>
@@ -1528,7 +1555,7 @@
       </c>
       <c r="K9" s="16"/>
     </row>
-    <row r="10" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="39.6" x14ac:dyDescent="0.35">
       <c r="A10" s="23" t="s">
         <v>14</v>
       </c>
@@ -1541,8 +1568,8 @@
       <c r="D10" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>41</v>
+      <c r="E10" s="18" t="s">
+        <v>205</v>
       </c>
       <c r="F10" s="20" t="s">
         <v>33</v>
@@ -1575,7 +1602,7 @@
         <v>44</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>45</v>
+        <v>206</v>
       </c>
       <c r="F11" s="20" t="s">
         <v>33</v>
@@ -1608,7 +1635,7 @@
         <v>48</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>45</v>
+        <v>206</v>
       </c>
       <c r="F12" s="20" t="s">
         <v>33</v>
@@ -1641,7 +1668,7 @@
         <v>51</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>52</v>
+        <v>207</v>
       </c>
       <c r="F13" s="20" t="s">
         <v>33</v>
@@ -1773,7 +1800,7 @@
         <v>65</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>66</v>
+        <v>208</v>
       </c>
       <c r="F17" s="20" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
Today I learned how to set up Ollama, use the OpenAI API, and analyze websites through web scraping.
</commit_message>
<xml_diff>
--- a/dsa_top_problems.xlsx
+++ b/dsa_top_problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sande\OneDrive\Desktop\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA55AEFD-1568-41B3-9F40-C1BCD2441CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD76AC04-C6B9-46BC-8396-B249D42C34C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="211">
   <si>
     <t>🚀  DSA Interview Prep — Top Company-Asked Problems</t>
   </si>
@@ -619,12 +619,6 @@
     <t>Focus on Medium first — 80% of real interviews</t>
   </si>
   <si>
-    <t>o</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
     <t>✅</t>
   </si>
   <si>
@@ -655,7 +649,16 @@
     <t>Expand Around Center (palindrome center expand)</t>
   </si>
   <si>
-    <t xml:space="preserve">Its Dificult problem for me to solve </t>
+    <t>using a nested loop to check every pair of numbers in the list, and returning the indices of the first pair whose sum equals the target.</t>
+  </si>
+  <si>
+    <t>keeps track of the lowest price seen so far, and updates the maximum profit whenever selling at the current price would give a better profit than previously recorded.</t>
+  </si>
+  <si>
+    <t>It iterates through prices once, tracking the minimum price so far and updating the maximum profit by comparing the current price minus that minimum.</t>
+  </si>
+  <si>
+    <t>It iterates through the array while tracking both the current maximum and minimum products (to handle negatives), updating them at each step and keeping the highest product found overall.</t>
   </si>
 </sst>
 </file>
@@ -1304,7 +1307,7 @@
     <col min="8" max="8" width="48" style="12" customWidth="1"/>
     <col min="9" max="9" width="10" style="12" customWidth="1"/>
     <col min="10" max="10" width="9" style="12" customWidth="1"/>
-    <col min="11" max="11" width="30.77734375" style="12" customWidth="1"/>
+    <col min="11" max="11" width="43.33203125" style="12" customWidth="1"/>
     <col min="12" max="16384" width="8.88671875" style="12"/>
   </cols>
   <sheetData>
@@ -1388,9 +1391,9 @@
       <c r="J4" s="25"/>
       <c r="K4" s="25"/>
     </row>
-    <row r="5" spans="1:11" ht="26.4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="52.8" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B5" s="13">
         <v>1</v>
@@ -1402,7 +1405,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>18</v>
@@ -1419,11 +1422,13 @@
       <c r="J5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="16"/>
-    </row>
-    <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K5" s="18" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="66" x14ac:dyDescent="0.35">
       <c r="A6" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B6" s="13">
         <v>2</v>
@@ -1435,7 +1440,7 @@
         <v>23</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>18</v>
@@ -1452,11 +1457,13 @@
       <c r="J6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="16"/>
+      <c r="K6" s="18" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="26.4" x14ac:dyDescent="0.35">
       <c r="A7" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B7" s="13">
         <v>3</v>
@@ -1468,7 +1475,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>18</v>
@@ -1480,10 +1487,10 @@
         <v>29</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>197</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>198</v>
+        <v>21</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>21</v>
       </c>
       <c r="K7" s="18"/>
     </row>
@@ -1501,7 +1508,7 @@
         <v>31</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F8" s="20" t="s">
         <v>33</v>
@@ -1518,13 +1525,11 @@
       <c r="J8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="16" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="33.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K8" s="16"/>
+    </row>
+    <row r="9" spans="1:11" ht="52.8" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B9" s="13">
         <v>5</v>
@@ -1536,7 +1541,7 @@
         <v>36</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F9" s="20" t="s">
         <v>33</v>
@@ -1553,11 +1558,13 @@
       <c r="J9" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K9" s="16"/>
-    </row>
-    <row r="10" spans="1:11" ht="39.6" x14ac:dyDescent="0.35">
+      <c r="K9" s="18" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="66" x14ac:dyDescent="0.35">
       <c r="A10" s="23" t="s">
-        <v>14</v>
+        <v>197</v>
       </c>
       <c r="B10" s="13">
         <v>6</v>
@@ -1569,7 +1576,7 @@
         <v>40</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F10" s="20" t="s">
         <v>33</v>
@@ -1586,7 +1593,9 @@
       <c r="J10" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K10" s="16"/>
+      <c r="K10" s="18" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="23" t="s">
@@ -1602,7 +1611,7 @@
         <v>44</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F11" s="20" t="s">
         <v>33</v>
@@ -1635,7 +1644,7 @@
         <v>48</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F12" s="20" t="s">
         <v>33</v>
@@ -1668,7 +1677,7 @@
         <v>51</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F13" s="20" t="s">
         <v>33</v>
@@ -1722,7 +1731,7 @@
     </row>
     <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B15" s="13">
         <v>11</v>
@@ -1800,7 +1809,7 @@
         <v>65</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F17" s="20" t="s">
         <v>33</v>

</xml_diff>